<commit_message>
Add folder scaffolding, README, .gitignore, data download docs
</commit_message>
<xml_diff>
--- a/Final Project/mediawave_timeline.xlsx
+++ b/Final Project/mediawave_timeline.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usfedu-my.sharepoint.com/personal/nganguyen_usf_edu/Documents/USF/Classes/Spring 2026/ISM4545/ism4545-data-avengers/Final Project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="31" documentId="11_695FBCD96809CC007B26151414FD1E818E5C6ACA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8AE70834-B17F-064C-8FC1-62EF80FA072A}"/>
+  <xr:revisionPtr revIDLastSave="33" documentId="11_695FBCD96809CC007B26151414FD1E818E5C6ACA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6489D001-5C9F-F74C-8369-EE408645A7B8}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17220" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,6 +18,9 @@
     <sheet name="Per-Person Summary" sheetId="3" r:id="rId3"/>
     <sheet name="Rubric Checklist" sheetId="4" r:id="rId4"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Daily Tasks'!$A$1:$G$111</definedName>
+  </definedNames>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -1610,6 +1613,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:G111"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
@@ -1645,7 +1649,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="6">
         <v>1</v>
       </c>
@@ -1683,7 +1687,7 @@
       <c r="F3" s="8"/>
       <c r="G3" s="8"/>
     </row>
-    <row r="4" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="6">
         <v>1</v>
       </c>
@@ -1702,7 +1706,7 @@
       <c r="F4" s="8"/>
       <c r="G4" s="8"/>
     </row>
-    <row r="5" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="6">
         <v>1</v>
       </c>
@@ -1721,7 +1725,7 @@
       <c r="F5" s="8"/>
       <c r="G5" s="8"/>
     </row>
-    <row r="6" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="6">
         <v>1</v>
       </c>
@@ -1740,7 +1744,7 @@
       <c r="F6" s="8"/>
       <c r="G6" s="8"/>
     </row>
-    <row r="7" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="6">
         <v>1</v>
       </c>
@@ -1759,7 +1763,7 @@
       <c r="F7" s="8"/>
       <c r="G7" s="8"/>
     </row>
-    <row r="8" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="6">
         <v>1</v>
       </c>
@@ -1778,7 +1782,7 @@
       <c r="F8" s="8"/>
       <c r="G8" s="8"/>
     </row>
-    <row r="9" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="6">
         <v>1</v>
       </c>
@@ -1797,7 +1801,7 @@
       <c r="F9" s="8"/>
       <c r="G9" s="8"/>
     </row>
-    <row r="10" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="6">
         <v>1</v>
       </c>
@@ -1816,7 +1820,7 @@
       <c r="F10" s="8"/>
       <c r="G10" s="8"/>
     </row>
-    <row r="11" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="6">
         <v>1</v>
       </c>
@@ -1835,7 +1839,7 @@
       <c r="F11" s="8"/>
       <c r="G11" s="8"/>
     </row>
-    <row r="12" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="6">
         <v>1</v>
       </c>
@@ -1854,7 +1858,7 @@
       <c r="F12" s="8"/>
       <c r="G12" s="8"/>
     </row>
-    <row r="13" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="6">
         <v>1</v>
       </c>
@@ -1873,7 +1877,7 @@
       <c r="F13" s="8"/>
       <c r="G13" s="8"/>
     </row>
-    <row r="14" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="6">
         <v>1</v>
       </c>
@@ -1892,7 +1896,7 @@
       <c r="F14" s="8"/>
       <c r="G14" s="8"/>
     </row>
-    <row r="15" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="6">
         <v>1</v>
       </c>
@@ -1911,7 +1915,7 @@
       <c r="F15" s="8"/>
       <c r="G15" s="8"/>
     </row>
-    <row r="16" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="6">
         <v>1</v>
       </c>
@@ -1930,7 +1934,7 @@
       <c r="F16" s="8"/>
       <c r="G16" s="8"/>
     </row>
-    <row r="17" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="6">
         <v>2</v>
       </c>
@@ -1949,7 +1953,7 @@
       <c r="F17" s="8"/>
       <c r="G17" s="8"/>
     </row>
-    <row r="18" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="6">
         <v>2</v>
       </c>
@@ -1968,7 +1972,7 @@
       <c r="F18" s="8"/>
       <c r="G18" s="8"/>
     </row>
-    <row r="19" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="6">
         <v>2</v>
       </c>
@@ -1987,7 +1991,7 @@
       <c r="F19" s="8"/>
       <c r="G19" s="8"/>
     </row>
-    <row r="20" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="6">
         <v>2</v>
       </c>
@@ -2006,7 +2010,7 @@
       <c r="F20" s="8"/>
       <c r="G20" s="8"/>
     </row>
-    <row r="21" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="6">
         <v>2</v>
       </c>
@@ -2025,7 +2029,7 @@
       <c r="F21" s="8"/>
       <c r="G21" s="8"/>
     </row>
-    <row r="22" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="6">
         <v>2</v>
       </c>
@@ -2044,7 +2048,7 @@
       <c r="F22" s="8"/>
       <c r="G22" s="8"/>
     </row>
-    <row r="23" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="6">
         <v>2</v>
       </c>
@@ -2063,7 +2067,7 @@
       <c r="F23" s="8"/>
       <c r="G23" s="8"/>
     </row>
-    <row r="24" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="6">
         <v>2</v>
       </c>
@@ -2082,7 +2086,7 @@
       <c r="F24" s="8"/>
       <c r="G24" s="8"/>
     </row>
-    <row r="25" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="6">
         <v>2</v>
       </c>
@@ -2101,7 +2105,7 @@
       <c r="F25" s="8"/>
       <c r="G25" s="8"/>
     </row>
-    <row r="26" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="6">
         <v>2</v>
       </c>
@@ -2120,7 +2124,7 @@
       <c r="F26" s="8"/>
       <c r="G26" s="8"/>
     </row>
-    <row r="27" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="6">
         <v>2</v>
       </c>
@@ -2139,7 +2143,7 @@
       <c r="F27" s="8"/>
       <c r="G27" s="8"/>
     </row>
-    <row r="28" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="6">
         <v>2</v>
       </c>
@@ -2158,7 +2162,7 @@
       <c r="F28" s="8"/>
       <c r="G28" s="8"/>
     </row>
-    <row r="29" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="6">
         <v>2</v>
       </c>
@@ -2215,7 +2219,7 @@
       <c r="F31" s="8"/>
       <c r="G31" s="8"/>
     </row>
-    <row r="32" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="6">
         <v>3</v>
       </c>
@@ -2234,7 +2238,7 @@
       <c r="F32" s="8"/>
       <c r="G32" s="8"/>
     </row>
-    <row r="33" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="6">
         <v>3</v>
       </c>
@@ -2253,7 +2257,7 @@
       <c r="F33" s="8"/>
       <c r="G33" s="8"/>
     </row>
-    <row r="34" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="6">
         <v>3</v>
       </c>
@@ -2272,7 +2276,7 @@
       <c r="F34" s="8"/>
       <c r="G34" s="8"/>
     </row>
-    <row r="35" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="6">
         <v>3</v>
       </c>
@@ -2291,7 +2295,7 @@
       <c r="F35" s="8"/>
       <c r="G35" s="8"/>
     </row>
-    <row r="36" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="6">
         <v>3</v>
       </c>
@@ -2310,7 +2314,7 @@
       <c r="F36" s="8"/>
       <c r="G36" s="8"/>
     </row>
-    <row r="37" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="6">
         <v>3</v>
       </c>
@@ -2329,7 +2333,7 @@
       <c r="F37" s="8"/>
       <c r="G37" s="8"/>
     </row>
-    <row r="38" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="6">
         <v>3</v>
       </c>
@@ -2348,7 +2352,7 @@
       <c r="F38" s="8"/>
       <c r="G38" s="8"/>
     </row>
-    <row r="39" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="6">
         <v>3</v>
       </c>
@@ -2367,7 +2371,7 @@
       <c r="F39" s="8"/>
       <c r="G39" s="8"/>
     </row>
-    <row r="40" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="6">
         <v>3</v>
       </c>
@@ -2386,7 +2390,7 @@
       <c r="F40" s="8"/>
       <c r="G40" s="8"/>
     </row>
-    <row r="41" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="6">
         <v>3</v>
       </c>
@@ -2405,7 +2409,7 @@
       <c r="F41" s="8"/>
       <c r="G41" s="8"/>
     </row>
-    <row r="42" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="6">
         <v>3</v>
       </c>
@@ -2424,7 +2428,7 @@
       <c r="F42" s="8"/>
       <c r="G42" s="8"/>
     </row>
-    <row r="43" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="6">
         <v>3</v>
       </c>
@@ -2443,7 +2447,7 @@
       <c r="F43" s="8"/>
       <c r="G43" s="8"/>
     </row>
-    <row r="44" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="6">
         <v>3</v>
       </c>
@@ -2462,7 +2466,7 @@
       <c r="F44" s="8"/>
       <c r="G44" s="8"/>
     </row>
-    <row r="45" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="6">
         <v>3</v>
       </c>
@@ -2481,7 +2485,7 @@
       <c r="F45" s="8"/>
       <c r="G45" s="8"/>
     </row>
-    <row r="46" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="6">
         <v>3</v>
       </c>
@@ -2538,7 +2542,7 @@
       <c r="F48" s="8"/>
       <c r="G48" s="8"/>
     </row>
-    <row r="49" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="6">
         <v>4</v>
       </c>
@@ -2557,7 +2561,7 @@
       <c r="F49" s="8"/>
       <c r="G49" s="8"/>
     </row>
-    <row r="50" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="6">
         <v>4</v>
       </c>
@@ -2576,7 +2580,7 @@
       <c r="F50" s="8"/>
       <c r="G50" s="8"/>
     </row>
-    <row r="51" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="6">
         <v>4</v>
       </c>
@@ -2595,7 +2599,7 @@
       <c r="F51" s="8"/>
       <c r="G51" s="8"/>
     </row>
-    <row r="52" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="6">
         <v>4</v>
       </c>
@@ -2614,7 +2618,7 @@
       <c r="F52" s="8"/>
       <c r="G52" s="8"/>
     </row>
-    <row r="53" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="6">
         <v>4</v>
       </c>
@@ -2633,7 +2637,7 @@
       <c r="F53" s="8"/>
       <c r="G53" s="8"/>
     </row>
-    <row r="54" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="6">
         <v>4</v>
       </c>
@@ -2652,7 +2656,7 @@
       <c r="F54" s="8"/>
       <c r="G54" s="8"/>
     </row>
-    <row r="55" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="6">
         <v>4</v>
       </c>
@@ -2671,7 +2675,7 @@
       <c r="F55" s="8"/>
       <c r="G55" s="8"/>
     </row>
-    <row r="56" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="6">
         <v>4</v>
       </c>
@@ -2690,7 +2694,7 @@
       <c r="F56" s="8"/>
       <c r="G56" s="8"/>
     </row>
-    <row r="57" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="6">
         <v>4</v>
       </c>
@@ -2709,7 +2713,7 @@
       <c r="F57" s="8"/>
       <c r="G57" s="8"/>
     </row>
-    <row r="58" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="6">
         <v>4</v>
       </c>
@@ -2728,7 +2732,7 @@
       <c r="F58" s="8"/>
       <c r="G58" s="8"/>
     </row>
-    <row r="59" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="6">
         <v>4</v>
       </c>
@@ -2785,7 +2789,7 @@
       <c r="F61" s="8"/>
       <c r="G61" s="8"/>
     </row>
-    <row r="62" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62" s="6">
         <v>5</v>
       </c>
@@ -2804,7 +2808,7 @@
       <c r="F62" s="8"/>
       <c r="G62" s="8"/>
     </row>
-    <row r="63" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" s="6">
         <v>5</v>
       </c>
@@ -2823,7 +2827,7 @@
       <c r="F63" s="8"/>
       <c r="G63" s="8"/>
     </row>
-    <row r="64" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" s="6">
         <v>5</v>
       </c>
@@ -2842,7 +2846,7 @@
       <c r="F64" s="8"/>
       <c r="G64" s="8"/>
     </row>
-    <row r="65" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A65" s="6">
         <v>5</v>
       </c>
@@ -2861,7 +2865,7 @@
       <c r="F65" s="8"/>
       <c r="G65" s="8"/>
     </row>
-    <row r="66" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A66" s="6">
         <v>5</v>
       </c>
@@ -2880,7 +2884,7 @@
       <c r="F66" s="8"/>
       <c r="G66" s="8"/>
     </row>
-    <row r="67" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A67" s="6">
         <v>5</v>
       </c>
@@ -2899,7 +2903,7 @@
       <c r="F67" s="8"/>
       <c r="G67" s="8"/>
     </row>
-    <row r="68" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A68" s="6">
         <v>5</v>
       </c>
@@ -2918,7 +2922,7 @@
       <c r="F68" s="8"/>
       <c r="G68" s="8"/>
     </row>
-    <row r="69" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A69" s="6">
         <v>5</v>
       </c>
@@ -2937,7 +2941,7 @@
       <c r="F69" s="8"/>
       <c r="G69" s="8"/>
     </row>
-    <row r="70" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A70" s="6">
         <v>5</v>
       </c>
@@ -2956,7 +2960,7 @@
       <c r="F70" s="8"/>
       <c r="G70" s="8"/>
     </row>
-    <row r="71" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A71" s="6">
         <v>5</v>
       </c>
@@ -2975,7 +2979,7 @@
       <c r="F71" s="8"/>
       <c r="G71" s="8"/>
     </row>
-    <row r="72" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A72" s="6">
         <v>5</v>
       </c>
@@ -2994,7 +2998,7 @@
       <c r="F72" s="8"/>
       <c r="G72" s="8"/>
     </row>
-    <row r="73" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A73" s="6">
         <v>5</v>
       </c>
@@ -3013,7 +3017,7 @@
       <c r="F73" s="8"/>
       <c r="G73" s="8"/>
     </row>
-    <row r="74" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A74" s="6">
         <v>5</v>
       </c>
@@ -3032,7 +3036,7 @@
       <c r="F74" s="8"/>
       <c r="G74" s="8"/>
     </row>
-    <row r="75" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A75" s="6">
         <v>5</v>
       </c>
@@ -3108,7 +3112,7 @@
       <c r="F78" s="8"/>
       <c r="G78" s="8"/>
     </row>
-    <row r="79" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A79" s="6">
         <v>6</v>
       </c>
@@ -3127,7 +3131,7 @@
       <c r="F79" s="8"/>
       <c r="G79" s="8"/>
     </row>
-    <row r="80" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A80" s="6">
         <v>6</v>
       </c>
@@ -3146,7 +3150,7 @@
       <c r="F80" s="8"/>
       <c r="G80" s="8"/>
     </row>
-    <row r="81" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A81" s="6">
         <v>6</v>
       </c>
@@ -3165,7 +3169,7 @@
       <c r="F81" s="8"/>
       <c r="G81" s="8"/>
     </row>
-    <row r="82" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A82" s="6">
         <v>6</v>
       </c>
@@ -3184,7 +3188,7 @@
       <c r="F82" s="8"/>
       <c r="G82" s="8"/>
     </row>
-    <row r="83" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A83" s="6">
         <v>6</v>
       </c>
@@ -3203,7 +3207,7 @@
       <c r="F83" s="8"/>
       <c r="G83" s="8"/>
     </row>
-    <row r="84" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A84" s="6">
         <v>6</v>
       </c>
@@ -3222,7 +3226,7 @@
       <c r="F84" s="8"/>
       <c r="G84" s="8"/>
     </row>
-    <row r="85" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A85" s="6">
         <v>6</v>
       </c>
@@ -3241,7 +3245,7 @@
       <c r="F85" s="8"/>
       <c r="G85" s="8"/>
     </row>
-    <row r="86" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A86" s="6">
         <v>6</v>
       </c>
@@ -3317,7 +3321,7 @@
       <c r="F89" s="8"/>
       <c r="G89" s="8"/>
     </row>
-    <row r="90" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A90" s="6">
         <v>7</v>
       </c>
@@ -3336,7 +3340,7 @@
       <c r="F90" s="8"/>
       <c r="G90" s="8"/>
     </row>
-    <row r="91" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A91" s="6">
         <v>7</v>
       </c>
@@ -3355,7 +3359,7 @@
       <c r="F91" s="8"/>
       <c r="G91" s="8"/>
     </row>
-    <row r="92" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A92" s="6">
         <v>7</v>
       </c>
@@ -3374,7 +3378,7 @@
       <c r="F92" s="8"/>
       <c r="G92" s="8"/>
     </row>
-    <row r="93" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A93" s="6">
         <v>7</v>
       </c>
@@ -3393,7 +3397,7 @@
       <c r="F93" s="8"/>
       <c r="G93" s="8"/>
     </row>
-    <row r="94" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A94" s="6">
         <v>7</v>
       </c>
@@ -3450,7 +3454,7 @@
       <c r="F96" s="8"/>
       <c r="G96" s="8"/>
     </row>
-    <row r="97" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A97" s="6">
         <v>8</v>
       </c>
@@ -3469,7 +3473,7 @@
       <c r="F97" s="8"/>
       <c r="G97" s="8"/>
     </row>
-    <row r="98" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A98" s="6">
         <v>8</v>
       </c>
@@ -3488,7 +3492,7 @@
       <c r="F98" s="8"/>
       <c r="G98" s="8"/>
     </row>
-    <row r="99" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A99" s="6">
         <v>8</v>
       </c>
@@ -3507,7 +3511,7 @@
       <c r="F99" s="8"/>
       <c r="G99" s="8"/>
     </row>
-    <row r="100" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A100" s="6">
         <v>8</v>
       </c>
@@ -3526,7 +3530,7 @@
       <c r="F100" s="8"/>
       <c r="G100" s="8"/>
     </row>
-    <row r="101" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A101" s="6">
         <v>8</v>
       </c>
@@ -3583,7 +3587,7 @@
       <c r="F103" s="8"/>
       <c r="G103" s="8"/>
     </row>
-    <row r="104" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A104" s="6">
         <v>8</v>
       </c>
@@ -3602,7 +3606,7 @@
       <c r="F104" s="8"/>
       <c r="G104" s="8"/>
     </row>
-    <row r="105" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A105" s="6">
         <v>9</v>
       </c>
@@ -3678,7 +3682,7 @@
       <c r="F108" s="8"/>
       <c r="G108" s="8"/>
     </row>
-    <row r="109" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A109" s="6">
         <v>12</v>
       </c>
@@ -3697,7 +3701,7 @@
       <c r="F109" s="8"/>
       <c r="G109" s="8"/>
     </row>
-    <row r="110" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A110" s="6">
         <v>13</v>
       </c>
@@ -3716,7 +3720,7 @@
       <c r="F110" s="8"/>
       <c r="G110" s="8"/>
     </row>
-    <row r="111" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A111" s="6">
         <v>13</v>
       </c>
@@ -3736,6 +3740,13 @@
       <c r="G111" s="8"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:G111" xr:uid="{00000000-0001-0000-0100-000000000000}">
+    <filterColumn colId="2">
+      <filters>
+        <filter val="Helen"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <conditionalFormatting sqref="F2:F111">
     <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
       <formula>"Done"</formula>

</xml_diff>

<commit_message>
Updated Helen's task status
</commit_message>
<xml_diff>
--- a/Final Project/mediawave_timeline.xlsx
+++ b/Final Project/mediawave_timeline.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usfedu-my.sharepoint.com/personal/nganguyen_usf_edu/Documents/USF/Classes/Spring 2026/ISM4545/ism4545-data-avengers/Final Project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="33" documentId="11_695FBCD96809CC007B26151414FD1E818E5C6ACA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6489D001-5C9F-F74C-8369-EE408645A7B8}"/>
+  <xr:revisionPtr revIDLastSave="34" documentId="11_695FBCD96809CC007B26151414FD1E818E5C6ACA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3658B40D-4E76-1D44-85D7-133CF67AD789}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17220" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="698" uniqueCount="270">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="699" uniqueCount="270">
   <si>
     <t>MediaWave Streaming — Final Project Timeline</t>
   </si>
@@ -1557,7 +1557,7 @@
       </c>
       <c r="B15" s="1">
         <f>COUNTIF('Daily Tasks'!F:F,"Done")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D15" s="35" t="s">
         <v>30</v>
@@ -1571,7 +1571,7 @@
       </c>
       <c r="B16" s="4">
         <f>IFERROR(B15/B14,0)</f>
-        <v>0</v>
+        <v>9.0909090909090905E-3</v>
       </c>
       <c r="D16" s="35" t="s">
         <v>32</v>
@@ -1684,7 +1684,9 @@
       <c r="E3" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="F3" s="8"/>
+      <c r="F3" s="8" t="s">
+        <v>184</v>
+      </c>
       <c r="G3" s="8"/>
     </row>
     <row r="4" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
@@ -3978,11 +3980,11 @@
       </c>
       <c r="D15" s="14">
         <f>COUNTIFS('Daily Tasks'!A:A,1,'Daily Tasks'!F:F,"Done")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E15" s="15">
         <f t="shared" ref="E15:E27" si="1">IFERROR(D15/C15,0)</f>
-        <v>0</v>
+        <v>6.6666666666666666E-2</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Updated the name for data-lake-architecture. 1st draft of exec report
</commit_message>
<xml_diff>
--- a/Final Project/mediawave_timeline.xlsx
+++ b/Final Project/mediawave_timeline.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usfedu-my.sharepoint.com/personal/nganguyen_usf_edu/Documents/USF/Classes/Spring 2026/ISM4545/ism4545-data-avengers/Final Project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="34" documentId="11_695FBCD96809CC007B26151414FD1E818E5C6ACA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3658B40D-4E76-1D44-85D7-133CF67AD789}"/>
+  <xr:revisionPtr revIDLastSave="41" documentId="11_695FBCD96809CC007B26151414FD1E818E5C6ACA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D41C614E-84DF-2044-8B6C-5E7ADA38450B}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17220" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="699" uniqueCount="270">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="701" uniqueCount="270">
   <si>
     <t>MediaWave Streaming — Final Project Timeline</t>
   </si>
@@ -338,9 +338,6 @@
     <t>Wire ingest, validate, clean tasks to real logic; allow 1-2h for Airflow↔Spark networking debugging</t>
   </si>
   <si>
-    <t>Update architecture diagram to reflect what A actually built</t>
-  </si>
-  <si>
     <t>Start collecting screenshots: HDFS UI with files, Spark UI with workers, Airflow DAG</t>
   </si>
   <si>
@@ -852,6 +849,9 @@
   </si>
   <si>
     <t>PM + Writer</t>
+  </si>
+  <si>
+    <t>Update architecture diagram to reflect what Juan actually built</t>
   </si>
 </sst>
 </file>
@@ -1024,7 +1024,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1100,6 +1100,9 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1442,7 +1445,7 @@
         <v>5</v>
       </c>
       <c r="D5" s="24" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>6</v>
@@ -1459,7 +1462,7 @@
         <v>9</v>
       </c>
       <c r="D6" s="25" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>10</v>
@@ -1476,7 +1479,7 @@
         <v>13</v>
       </c>
       <c r="D7" s="26" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>14</v>
@@ -1493,7 +1496,7 @@
         <v>17</v>
       </c>
       <c r="D8" s="27" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>18</v>
@@ -1510,10 +1513,10 @@
         <v>21</v>
       </c>
       <c r="D9" s="28" t="s">
+        <v>267</v>
+      </c>
+      <c r="E9" s="29" t="s">
         <v>268</v>
-      </c>
-      <c r="E9" s="29" t="s">
-        <v>269</v>
       </c>
       <c r="F9" s="3" t="s">
         <v>23</v>
@@ -1557,7 +1560,7 @@
       </c>
       <c r="B15" s="1">
         <f>COUNTIF('Daily Tasks'!F:F,"Done")</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D15" s="35" t="s">
         <v>30</v>
@@ -1571,7 +1574,7 @@
       </c>
       <c r="B16" s="4">
         <f>IFERROR(B15/B14,0)</f>
-        <v>9.0909090909090905E-3</v>
+        <v>2.7272727272727271E-2</v>
       </c>
       <c r="D16" s="35" t="s">
         <v>32</v>
@@ -1613,7 +1616,6 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:G111"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
@@ -1649,12 +1651,12 @@
         <v>41</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="6">
         <v>1</v>
       </c>
       <c r="B2" s="23" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="C2" s="7" t="s">
         <v>43</v>
@@ -1665,7 +1667,9 @@
       <c r="E2" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="F2" s="8"/>
+      <c r="F2" s="8" t="s">
+        <v>183</v>
+      </c>
       <c r="G2" s="8"/>
     </row>
     <row r="3" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -1676,7 +1680,7 @@
         <v>42</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="D3" s="8" t="s">
         <v>46</v>
@@ -1685,11 +1689,11 @@
         <v>47</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="G3" s="8"/>
     </row>
-    <row r="4" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="6">
         <v>1</v>
       </c>
@@ -1697,7 +1701,7 @@
         <v>42</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="D4" s="8" t="s">
         <v>48</v>
@@ -1708,7 +1712,7 @@
       <c r="F4" s="8"/>
       <c r="G4" s="8"/>
     </row>
-    <row r="5" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="6">
         <v>1</v>
       </c>
@@ -1716,7 +1720,7 @@
         <v>42</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="D5" s="8" t="s">
         <v>48</v>
@@ -1727,7 +1731,7 @@
       <c r="F5" s="8"/>
       <c r="G5" s="8"/>
     </row>
-    <row r="6" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="6">
         <v>1</v>
       </c>
@@ -1735,7 +1739,7 @@
         <v>42</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="D6" s="8" t="s">
         <v>51</v>
@@ -1746,7 +1750,7 @@
       <c r="F6" s="8"/>
       <c r="G6" s="8"/>
     </row>
-    <row r="7" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="6">
         <v>1</v>
       </c>
@@ -1754,7 +1758,7 @@
         <v>42</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="D7" s="8" t="s">
         <v>51</v>
@@ -1765,7 +1769,7 @@
       <c r="F7" s="8"/>
       <c r="G7" s="8"/>
     </row>
-    <row r="8" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="6">
         <v>1</v>
       </c>
@@ -1773,7 +1777,7 @@
         <v>42</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="D8" s="8" t="s">
         <v>51</v>
@@ -1784,7 +1788,7 @@
       <c r="F8" s="8"/>
       <c r="G8" s="8"/>
     </row>
-    <row r="9" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="6">
         <v>1</v>
       </c>
@@ -1792,7 +1796,7 @@
         <v>42</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="D9" s="8" t="s">
         <v>51</v>
@@ -1803,7 +1807,7 @@
       <c r="F9" s="8"/>
       <c r="G9" s="8"/>
     </row>
-    <row r="10" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="6">
         <v>1</v>
       </c>
@@ -1811,7 +1815,7 @@
         <v>42</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="D10" s="8" t="s">
         <v>51</v>
@@ -1822,7 +1826,7 @@
       <c r="F10" s="8"/>
       <c r="G10" s="8"/>
     </row>
-    <row r="11" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="6">
         <v>1</v>
       </c>
@@ -1830,7 +1834,7 @@
         <v>42</v>
       </c>
       <c r="C11" s="12" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="D11" s="8" t="s">
         <v>57</v>
@@ -1841,7 +1845,7 @@
       <c r="F11" s="8"/>
       <c r="G11" s="8"/>
     </row>
-    <row r="12" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="6">
         <v>1</v>
       </c>
@@ -1849,7 +1853,7 @@
         <v>42</v>
       </c>
       <c r="C12" s="12" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="D12" s="8" t="s">
         <v>57</v>
@@ -1860,7 +1864,7 @@
       <c r="F12" s="8"/>
       <c r="G12" s="8"/>
     </row>
-    <row r="13" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="6">
         <v>1</v>
       </c>
@@ -1868,7 +1872,7 @@
         <v>42</v>
       </c>
       <c r="C13" s="12" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="D13" s="8" t="s">
         <v>57</v>
@@ -1879,7 +1883,7 @@
       <c r="F13" s="8"/>
       <c r="G13" s="8"/>
     </row>
-    <row r="14" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="6">
         <v>1</v>
       </c>
@@ -1887,7 +1891,7 @@
         <v>42</v>
       </c>
       <c r="C14" s="13" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="D14" s="8" t="s">
         <v>61</v>
@@ -1898,7 +1902,7 @@
       <c r="F14" s="8"/>
       <c r="G14" s="8"/>
     </row>
-    <row r="15" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="6">
         <v>1</v>
       </c>
@@ -1906,7 +1910,7 @@
         <v>42</v>
       </c>
       <c r="C15" s="13" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="D15" s="8" t="s">
         <v>61</v>
@@ -1917,7 +1921,7 @@
       <c r="F15" s="8"/>
       <c r="G15" s="8"/>
     </row>
-    <row r="16" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="6">
         <v>1</v>
       </c>
@@ -1925,7 +1929,7 @@
         <v>42</v>
       </c>
       <c r="C16" s="13" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="D16" s="8" t="s">
         <v>61</v>
@@ -1936,7 +1940,7 @@
       <c r="F16" s="8"/>
       <c r="G16" s="8"/>
     </row>
-    <row r="17" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="6">
         <v>2</v>
       </c>
@@ -1944,7 +1948,7 @@
         <v>65</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="D17" s="8" t="s">
         <v>48</v>
@@ -1955,7 +1959,7 @@
       <c r="F17" s="8"/>
       <c r="G17" s="8"/>
     </row>
-    <row r="18" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="6">
         <v>2</v>
       </c>
@@ -1963,7 +1967,7 @@
         <v>65</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="D18" s="8" t="s">
         <v>48</v>
@@ -1974,7 +1978,7 @@
       <c r="F18" s="8"/>
       <c r="G18" s="8"/>
     </row>
-    <row r="19" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="6">
         <v>2</v>
       </c>
@@ -1982,7 +1986,7 @@
         <v>65</v>
       </c>
       <c r="C19" s="10" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="D19" s="8" t="s">
         <v>48</v>
@@ -1993,7 +1997,7 @@
       <c r="F19" s="8"/>
       <c r="G19" s="8"/>
     </row>
-    <row r="20" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="6">
         <v>2</v>
       </c>
@@ -2001,7 +2005,7 @@
         <v>65</v>
       </c>
       <c r="C20" s="10" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="D20" s="8" t="s">
         <v>48</v>
@@ -2012,7 +2016,7 @@
       <c r="F20" s="8"/>
       <c r="G20" s="8"/>
     </row>
-    <row r="21" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="6">
         <v>2</v>
       </c>
@@ -2020,7 +2024,7 @@
         <v>65</v>
       </c>
       <c r="C21" s="11" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="D21" s="8" t="s">
         <v>51</v>
@@ -2031,7 +2035,7 @@
       <c r="F21" s="8"/>
       <c r="G21" s="8"/>
     </row>
-    <row r="22" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="6">
         <v>2</v>
       </c>
@@ -2039,7 +2043,7 @@
         <v>65</v>
       </c>
       <c r="C22" s="11" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="D22" s="8" t="s">
         <v>51</v>
@@ -2050,7 +2054,7 @@
       <c r="F22" s="8"/>
       <c r="G22" s="8"/>
     </row>
-    <row r="23" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="6">
         <v>2</v>
       </c>
@@ -2058,7 +2062,7 @@
         <v>65</v>
       </c>
       <c r="C23" s="11" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="D23" s="8" t="s">
         <v>51</v>
@@ -2069,7 +2073,7 @@
       <c r="F23" s="8"/>
       <c r="G23" s="8"/>
     </row>
-    <row r="24" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="6">
         <v>2</v>
       </c>
@@ -2077,7 +2081,7 @@
         <v>65</v>
       </c>
       <c r="C24" s="11" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="D24" s="8" t="s">
         <v>51</v>
@@ -2088,7 +2092,7 @@
       <c r="F24" s="8"/>
       <c r="G24" s="8"/>
     </row>
-    <row r="25" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="6">
         <v>2</v>
       </c>
@@ -2096,7 +2100,7 @@
         <v>65</v>
       </c>
       <c r="C25" s="12" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="D25" s="8" t="s">
         <v>57</v>
@@ -2107,7 +2111,7 @@
       <c r="F25" s="8"/>
       <c r="G25" s="8"/>
     </row>
-    <row r="26" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="6">
         <v>2</v>
       </c>
@@ -2115,7 +2119,7 @@
         <v>65</v>
       </c>
       <c r="C26" s="12" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="D26" s="8" t="s">
         <v>57</v>
@@ -2126,7 +2130,7 @@
       <c r="F26" s="8"/>
       <c r="G26" s="8"/>
     </row>
-    <row r="27" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="6">
         <v>2</v>
       </c>
@@ -2134,7 +2138,7 @@
         <v>65</v>
       </c>
       <c r="C27" s="13" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="D27" s="8" t="s">
         <v>61</v>
@@ -2145,7 +2149,7 @@
       <c r="F27" s="8"/>
       <c r="G27" s="8"/>
     </row>
-    <row r="28" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="6">
         <v>2</v>
       </c>
@@ -2153,7 +2157,7 @@
         <v>65</v>
       </c>
       <c r="C28" s="13" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="D28" s="8" t="s">
         <v>61</v>
@@ -2164,7 +2168,7 @@
       <c r="F28" s="8"/>
       <c r="G28" s="8"/>
     </row>
-    <row r="29" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="6">
         <v>2</v>
       </c>
@@ -2172,7 +2176,7 @@
         <v>65</v>
       </c>
       <c r="C29" s="13" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="D29" s="8" t="s">
         <v>61</v>
@@ -2190,13 +2194,13 @@
       <c r="B30" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="C30" s="9" t="s">
-        <v>268</v>
+      <c r="C30" s="10" t="s">
+        <v>263</v>
       </c>
       <c r="D30" s="8" t="s">
         <v>79</v>
       </c>
-      <c r="E30" s="8" t="s">
+      <c r="E30" s="41" t="s">
         <v>80</v>
       </c>
       <c r="F30" s="8"/>
@@ -2210,7 +2214,7 @@
         <v>65</v>
       </c>
       <c r="C31" s="9" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="D31" s="8" t="s">
         <v>79</v>
@@ -2218,10 +2222,12 @@
       <c r="E31" s="8" t="s">
         <v>81</v>
       </c>
-      <c r="F31" s="8"/>
+      <c r="F31" s="8" t="s">
+        <v>183</v>
+      </c>
       <c r="G31" s="8"/>
     </row>
-    <row r="32" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="6">
         <v>3</v>
       </c>
@@ -2229,7 +2235,7 @@
         <v>82</v>
       </c>
       <c r="C32" s="10" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="D32" s="8" t="s">
         <v>48</v>
@@ -2240,7 +2246,7 @@
       <c r="F32" s="8"/>
       <c r="G32" s="8"/>
     </row>
-    <row r="33" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="6">
         <v>3</v>
       </c>
@@ -2248,7 +2254,7 @@
         <v>82</v>
       </c>
       <c r="C33" s="10" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="D33" s="8" t="s">
         <v>48</v>
@@ -2259,7 +2265,7 @@
       <c r="F33" s="8"/>
       <c r="G33" s="8"/>
     </row>
-    <row r="34" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="6">
         <v>3</v>
       </c>
@@ -2267,7 +2273,7 @@
         <v>82</v>
       </c>
       <c r="C34" s="10" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="D34" s="8" t="s">
         <v>48</v>
@@ -2278,7 +2284,7 @@
       <c r="F34" s="8"/>
       <c r="G34" s="8"/>
     </row>
-    <row r="35" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="6">
         <v>3</v>
       </c>
@@ -2286,7 +2292,7 @@
         <v>82</v>
       </c>
       <c r="C35" s="10" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="D35" s="8" t="s">
         <v>48</v>
@@ -2297,7 +2303,7 @@
       <c r="F35" s="8"/>
       <c r="G35" s="8"/>
     </row>
-    <row r="36" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="6">
         <v>3</v>
       </c>
@@ -2305,7 +2311,7 @@
         <v>82</v>
       </c>
       <c r="C36" s="10" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="D36" s="8" t="s">
         <v>48</v>
@@ -2316,7 +2322,7 @@
       <c r="F36" s="8"/>
       <c r="G36" s="8"/>
     </row>
-    <row r="37" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="6">
         <v>3</v>
       </c>
@@ -2324,7 +2330,7 @@
         <v>82</v>
       </c>
       <c r="C37" s="10" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="D37" s="8" t="s">
         <v>48</v>
@@ -2335,7 +2341,7 @@
       <c r="F37" s="8"/>
       <c r="G37" s="8"/>
     </row>
-    <row r="38" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="6">
         <v>3</v>
       </c>
@@ -2343,7 +2349,7 @@
         <v>82</v>
       </c>
       <c r="C38" s="11" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="D38" s="8" t="s">
         <v>51</v>
@@ -2354,7 +2360,7 @@
       <c r="F38" s="8"/>
       <c r="G38" s="8"/>
     </row>
-    <row r="39" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="6">
         <v>3</v>
       </c>
@@ -2362,7 +2368,7 @@
         <v>82</v>
       </c>
       <c r="C39" s="11" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="D39" s="8" t="s">
         <v>51</v>
@@ -2373,7 +2379,7 @@
       <c r="F39" s="8"/>
       <c r="G39" s="8"/>
     </row>
-    <row r="40" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="6">
         <v>3</v>
       </c>
@@ -2381,7 +2387,7 @@
         <v>82</v>
       </c>
       <c r="C40" s="11" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="D40" s="8" t="s">
         <v>51</v>
@@ -2392,7 +2398,7 @@
       <c r="F40" s="8"/>
       <c r="G40" s="8"/>
     </row>
-    <row r="41" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="6">
         <v>3</v>
       </c>
@@ -2400,7 +2406,7 @@
         <v>82</v>
       </c>
       <c r="C41" s="11" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="D41" s="8" t="s">
         <v>51</v>
@@ -2411,7 +2417,7 @@
       <c r="F41" s="8"/>
       <c r="G41" s="8"/>
     </row>
-    <row r="42" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="6">
         <v>3</v>
       </c>
@@ -2419,7 +2425,7 @@
         <v>82</v>
       </c>
       <c r="C42" s="12" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="D42" s="8" t="s">
         <v>57</v>
@@ -2430,7 +2436,7 @@
       <c r="F42" s="8"/>
       <c r="G42" s="8"/>
     </row>
-    <row r="43" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="6">
         <v>3</v>
       </c>
@@ -2438,7 +2444,7 @@
         <v>82</v>
       </c>
       <c r="C43" s="12" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="D43" s="8" t="s">
         <v>57</v>
@@ -2449,7 +2455,7 @@
       <c r="F43" s="8"/>
       <c r="G43" s="8"/>
     </row>
-    <row r="44" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="6">
         <v>3</v>
       </c>
@@ -2457,7 +2463,7 @@
         <v>82</v>
       </c>
       <c r="C44" s="12" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="D44" s="8" t="s">
         <v>57</v>
@@ -2468,7 +2474,7 @@
       <c r="F44" s="8"/>
       <c r="G44" s="8"/>
     </row>
-    <row r="45" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="6">
         <v>3</v>
       </c>
@@ -2476,7 +2482,7 @@
         <v>82</v>
       </c>
       <c r="C45" s="13" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="D45" s="8" t="s">
         <v>61</v>
@@ -2487,7 +2493,7 @@
       <c r="F45" s="8"/>
       <c r="G45" s="8"/>
     </row>
-    <row r="46" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="6">
         <v>3</v>
       </c>
@@ -2495,7 +2501,7 @@
         <v>82</v>
       </c>
       <c r="C46" s="13" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="D46" s="8" t="s">
         <v>61</v>
@@ -2514,13 +2520,13 @@
         <v>82</v>
       </c>
       <c r="C47" s="9" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="D47" s="8" t="s">
         <v>79</v>
       </c>
-      <c r="E47" s="8" t="s">
-        <v>98</v>
+      <c r="E47" s="41" t="s">
+        <v>269</v>
       </c>
       <c r="F47" s="8"/>
       <c r="G47" s="8"/>
@@ -2533,222 +2539,222 @@
         <v>82</v>
       </c>
       <c r="C48" s="9" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="D48" s="8" t="s">
         <v>79</v>
       </c>
       <c r="E48" s="8" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="F48" s="8"/>
       <c r="G48" s="8"/>
     </row>
-    <row r="49" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="6">
         <v>4</v>
       </c>
       <c r="B49" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="C49" s="10" t="s">
+        <v>263</v>
+      </c>
+      <c r="D49" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="C49" s="10" t="s">
-        <v>264</v>
-      </c>
-      <c r="D49" s="8" t="s">
+      <c r="E49" s="8" t="s">
         <v>101</v>
-      </c>
-      <c r="E49" s="8" t="s">
-        <v>102</v>
       </c>
       <c r="F49" s="8"/>
       <c r="G49" s="8"/>
     </row>
-    <row r="50" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="6">
         <v>4</v>
       </c>
       <c r="B50" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="C50" s="10" t="s">
+        <v>263</v>
+      </c>
+      <c r="D50" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="C50" s="10" t="s">
-        <v>264</v>
-      </c>
-      <c r="D50" s="8" t="s">
-        <v>101</v>
-      </c>
       <c r="E50" s="8" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F50" s="8"/>
       <c r="G50" s="8"/>
     </row>
-    <row r="51" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="6">
         <v>4</v>
       </c>
       <c r="B51" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C51" s="11" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="D51" s="8" t="s">
         <v>51</v>
       </c>
       <c r="E51" s="8" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F51" s="8"/>
       <c r="G51" s="8"/>
     </row>
-    <row r="52" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="6">
         <v>4</v>
       </c>
       <c r="B52" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C52" s="11" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="D52" s="8" t="s">
         <v>51</v>
       </c>
       <c r="E52" s="8" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="F52" s="8"/>
       <c r="G52" s="8"/>
     </row>
-    <row r="53" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="6">
         <v>4</v>
       </c>
       <c r="B53" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C53" s="11" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="D53" s="8" t="s">
         <v>51</v>
       </c>
       <c r="E53" s="8" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F53" s="8"/>
       <c r="G53" s="8"/>
     </row>
-    <row r="54" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="6">
         <v>4</v>
       </c>
       <c r="B54" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C54" s="11" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="D54" s="8" t="s">
         <v>51</v>
       </c>
       <c r="E54" s="8" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F54" s="8"/>
       <c r="G54" s="8"/>
     </row>
-    <row r="55" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="6">
         <v>4</v>
       </c>
       <c r="B55" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C55" s="11" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="D55" s="8" t="s">
         <v>51</v>
       </c>
       <c r="E55" s="8" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F55" s="8"/>
       <c r="G55" s="8"/>
     </row>
-    <row r="56" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="6">
         <v>4</v>
       </c>
       <c r="B56" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C56" s="12" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="D56" s="8" t="s">
         <v>57</v>
       </c>
       <c r="E56" s="8" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F56" s="8"/>
       <c r="G56" s="8"/>
     </row>
-    <row r="57" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="6">
         <v>4</v>
       </c>
       <c r="B57" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C57" s="12" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="D57" s="8" t="s">
         <v>57</v>
       </c>
       <c r="E57" s="8" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F57" s="8"/>
       <c r="G57" s="8"/>
     </row>
-    <row r="58" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="6">
         <v>4</v>
       </c>
       <c r="B58" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C58" s="13" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="D58" s="8" t="s">
         <v>61</v>
       </c>
       <c r="E58" s="8" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F58" s="8"/>
       <c r="G58" s="8"/>
     </row>
-    <row r="59" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="6">
         <v>4</v>
       </c>
       <c r="B59" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C59" s="13" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="D59" s="8" t="s">
         <v>61</v>
       </c>
       <c r="E59" s="8" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F59" s="8"/>
       <c r="G59" s="8"/>
@@ -2758,16 +2764,16 @@
         <v>4</v>
       </c>
       <c r="B60" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C60" s="9" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="D60" s="8" t="s">
         <v>79</v>
       </c>
       <c r="E60" s="8" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F60" s="8"/>
       <c r="G60" s="8"/>
@@ -2777,282 +2783,282 @@
         <v>4</v>
       </c>
       <c r="B61" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C61" s="9" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="D61" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="E61" s="8" t="s">
         <v>114</v>
-      </c>
-      <c r="E61" s="8" t="s">
-        <v>115</v>
       </c>
       <c r="F61" s="8"/>
       <c r="G61" s="8"/>
     </row>
-    <row r="62" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62" s="6">
         <v>5</v>
       </c>
       <c r="B62" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="C62" s="10" t="s">
+        <v>263</v>
+      </c>
+      <c r="D62" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="E62" s="8" t="s">
         <v>116</v>
-      </c>
-      <c r="C62" s="10" t="s">
-        <v>264</v>
-      </c>
-      <c r="D62" s="8" t="s">
-        <v>101</v>
-      </c>
-      <c r="E62" s="8" t="s">
-        <v>117</v>
       </c>
       <c r="F62" s="8"/>
       <c r="G62" s="8"/>
     </row>
-    <row r="63" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" s="6">
         <v>5</v>
       </c>
       <c r="B63" s="6" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C63" s="10" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="D63" s="8" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E63" s="8" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F63" s="8"/>
       <c r="G63" s="8"/>
     </row>
-    <row r="64" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" s="6">
         <v>5</v>
       </c>
       <c r="B64" s="6" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C64" s="10" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="D64" s="8" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E64" s="8" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F64" s="8"/>
       <c r="G64" s="8"/>
     </row>
-    <row r="65" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A65" s="6">
         <v>5</v>
       </c>
       <c r="B65" s="6" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C65" s="11" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="D65" s="8" t="s">
         <v>51</v>
       </c>
       <c r="E65" s="8" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F65" s="8"/>
       <c r="G65" s="8"/>
     </row>
-    <row r="66" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A66" s="6">
         <v>5</v>
       </c>
       <c r="B66" s="6" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C66" s="11" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="D66" s="8" t="s">
         <v>51</v>
       </c>
       <c r="E66" s="8" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F66" s="8"/>
       <c r="G66" s="8"/>
     </row>
-    <row r="67" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A67" s="6">
         <v>5</v>
       </c>
       <c r="B67" s="6" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C67" s="11" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="D67" s="8" t="s">
         <v>51</v>
       </c>
       <c r="E67" s="8" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F67" s="8"/>
       <c r="G67" s="8"/>
     </row>
-    <row r="68" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A68" s="6">
         <v>5</v>
       </c>
       <c r="B68" s="6" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C68" s="11" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="D68" s="8" t="s">
         <v>51</v>
       </c>
       <c r="E68" s="8" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="F68" s="8"/>
       <c r="G68" s="8"/>
     </row>
-    <row r="69" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A69" s="6">
         <v>5</v>
       </c>
       <c r="B69" s="6" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C69" s="12" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="D69" s="8" t="s">
         <v>57</v>
       </c>
       <c r="E69" s="8" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F69" s="8"/>
       <c r="G69" s="8"/>
     </row>
-    <row r="70" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A70" s="6">
         <v>5</v>
       </c>
       <c r="B70" s="6" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C70" s="12" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="D70" s="8" t="s">
         <v>57</v>
       </c>
       <c r="E70" s="8" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F70" s="8"/>
       <c r="G70" s="8"/>
     </row>
-    <row r="71" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A71" s="6">
         <v>5</v>
       </c>
       <c r="B71" s="6" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C71" s="12" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="D71" s="8" t="s">
         <v>57</v>
       </c>
       <c r="E71" s="8" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F71" s="8"/>
       <c r="G71" s="8"/>
     </row>
-    <row r="72" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A72" s="6">
         <v>5</v>
       </c>
       <c r="B72" s="6" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C72" s="13" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="D72" s="8" t="s">
         <v>61</v>
       </c>
       <c r="E72" s="8" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F72" s="8"/>
       <c r="G72" s="8"/>
     </row>
-    <row r="73" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A73" s="6">
         <v>5</v>
       </c>
       <c r="B73" s="6" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C73" s="13" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="D73" s="8" t="s">
         <v>61</v>
       </c>
       <c r="E73" s="8" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F73" s="8"/>
       <c r="G73" s="8"/>
     </row>
-    <row r="74" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A74" s="6">
         <v>5</v>
       </c>
       <c r="B74" s="6" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C74" s="13" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="D74" s="8" t="s">
         <v>61</v>
       </c>
       <c r="E74" s="8" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="F74" s="8"/>
       <c r="G74" s="8"/>
     </row>
-    <row r="75" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A75" s="6">
         <v>5</v>
       </c>
       <c r="B75" s="6" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C75" s="13" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="D75" s="8" t="s">
         <v>61</v>
       </c>
       <c r="E75" s="8" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F75" s="8"/>
       <c r="G75" s="8"/>
@@ -3062,16 +3068,16 @@
         <v>5</v>
       </c>
       <c r="B76" s="6" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C76" s="9" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="D76" s="8" t="s">
         <v>79</v>
       </c>
       <c r="E76" s="8" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F76" s="8"/>
       <c r="G76" s="8"/>
@@ -3081,16 +3087,16 @@
         <v>5</v>
       </c>
       <c r="B77" s="6" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C77" s="9" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="D77" s="8" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E77" s="8" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F77" s="8"/>
       <c r="G77" s="8"/>
@@ -3100,168 +3106,168 @@
         <v>5</v>
       </c>
       <c r="B78" s="6" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C78" s="9" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="D78" s="8" t="s">
         <v>79</v>
       </c>
       <c r="E78" s="8" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="F78" s="8"/>
       <c r="G78" s="8"/>
     </row>
-    <row r="79" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A79" s="6">
         <v>6</v>
       </c>
       <c r="B79" s="6" t="s">
+        <v>133</v>
+      </c>
+      <c r="C79" s="10" t="s">
+        <v>263</v>
+      </c>
+      <c r="D79" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="E79" s="8" t="s">
         <v>134</v>
-      </c>
-      <c r="C79" s="10" t="s">
-        <v>264</v>
-      </c>
-      <c r="D79" s="8" t="s">
-        <v>101</v>
-      </c>
-      <c r="E79" s="8" t="s">
-        <v>135</v>
       </c>
       <c r="F79" s="8"/>
       <c r="G79" s="8"/>
     </row>
-    <row r="80" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A80" s="6">
         <v>6</v>
       </c>
       <c r="B80" s="6" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C80" s="10" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="D80" s="8" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E80" s="8" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F80" s="8"/>
       <c r="G80" s="8"/>
     </row>
-    <row r="81" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A81" s="6">
         <v>6</v>
       </c>
       <c r="B81" s="6" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C81" s="11" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="D81" s="8" t="s">
         <v>51</v>
       </c>
       <c r="E81" s="8" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F81" s="8"/>
       <c r="G81" s="8"/>
     </row>
-    <row r="82" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A82" s="6">
         <v>6</v>
       </c>
       <c r="B82" s="6" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C82" s="11" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="D82" s="8" t="s">
         <v>51</v>
       </c>
       <c r="E82" s="8" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F82" s="8"/>
       <c r="G82" s="8"/>
     </row>
-    <row r="83" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A83" s="6">
         <v>6</v>
       </c>
       <c r="B83" s="6" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C83" s="11" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="D83" s="8" t="s">
+        <v>138</v>
+      </c>
+      <c r="E83" s="8" t="s">
         <v>139</v>
-      </c>
-      <c r="E83" s="8" t="s">
-        <v>140</v>
       </c>
       <c r="F83" s="8"/>
       <c r="G83" s="8"/>
     </row>
-    <row r="84" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A84" s="6">
         <v>6</v>
       </c>
       <c r="B84" s="6" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C84" s="12" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="D84" s="8" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="E84" s="8" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F84" s="8"/>
       <c r="G84" s="8"/>
     </row>
-    <row r="85" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A85" s="6">
         <v>6</v>
       </c>
       <c r="B85" s="6" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C85" s="12" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="D85" s="8" t="s">
         <v>57</v>
       </c>
       <c r="E85" s="8" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="F85" s="8"/>
       <c r="G85" s="8"/>
     </row>
-    <row r="86" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A86" s="6">
         <v>6</v>
       </c>
       <c r="B86" s="6" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C86" s="13" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="D86" s="8" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="E86" s="8" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="F86" s="8"/>
       <c r="G86" s="8"/>
@@ -3271,16 +3277,16 @@
         <v>6</v>
       </c>
       <c r="B87" s="6" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C87" s="9" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="D87" s="8" t="s">
         <v>79</v>
       </c>
       <c r="E87" s="8" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="F87" s="8"/>
       <c r="G87" s="8"/>
@@ -3290,16 +3296,16 @@
         <v>6</v>
       </c>
       <c r="B88" s="6" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C88" s="9" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="D88" s="8" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E88" s="8" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F88" s="8"/>
       <c r="G88" s="8"/>
@@ -3309,111 +3315,111 @@
         <v>6</v>
       </c>
       <c r="B89" s="6" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C89" s="9" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="D89" s="8" t="s">
+        <v>145</v>
+      </c>
+      <c r="E89" s="8" t="s">
         <v>146</v>
-      </c>
-      <c r="E89" s="8" t="s">
-        <v>147</v>
       </c>
       <c r="F89" s="8"/>
       <c r="G89" s="8"/>
     </row>
-    <row r="90" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A90" s="6">
         <v>7</v>
       </c>
       <c r="B90" s="6" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C90" s="7" t="s">
         <v>43</v>
       </c>
       <c r="D90" s="8" t="s">
+        <v>148</v>
+      </c>
+      <c r="E90" s="8" t="s">
         <v>149</v>
-      </c>
-      <c r="E90" s="8" t="s">
-        <v>150</v>
       </c>
       <c r="F90" s="8"/>
       <c r="G90" s="8"/>
     </row>
-    <row r="91" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A91" s="6">
         <v>7</v>
       </c>
       <c r="B91" s="6" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C91" s="10" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="D91" s="8" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E91" s="8" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="F91" s="8"/>
       <c r="G91" s="8"/>
     </row>
-    <row r="92" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A92" s="6">
         <v>7</v>
       </c>
       <c r="B92" s="6" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C92" s="11" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="D92" s="8" t="s">
         <v>51</v>
       </c>
       <c r="E92" s="8" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F92" s="8"/>
       <c r="G92" s="8"/>
     </row>
-    <row r="93" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A93" s="6">
         <v>7</v>
       </c>
       <c r="B93" s="6" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C93" s="12" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="D93" s="8" t="s">
         <v>57</v>
       </c>
       <c r="E93" s="8" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="F93" s="8"/>
       <c r="G93" s="8"/>
     </row>
-    <row r="94" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A94" s="6">
         <v>7</v>
       </c>
       <c r="B94" s="6" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C94" s="13" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="D94" s="8" t="s">
         <v>61</v>
       </c>
       <c r="E94" s="8" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="F94" s="8"/>
       <c r="G94" s="8"/>
@@ -3423,16 +3429,16 @@
         <v>7</v>
       </c>
       <c r="B95" s="6" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C95" s="9" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="D95" s="8" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="E95" s="8" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="F95" s="8"/>
       <c r="G95" s="8"/>
@@ -3442,111 +3448,111 @@
         <v>7</v>
       </c>
       <c r="B96" s="6" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C96" s="9" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="D96" s="8" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="E96" s="8" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="F96" s="8"/>
       <c r="G96" s="8"/>
     </row>
-    <row r="97" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A97" s="6">
         <v>8</v>
       </c>
       <c r="B97" s="6" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C97" s="7" t="s">
         <v>43</v>
       </c>
       <c r="D97" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="E97" s="8" t="s">
         <v>158</v>
-      </c>
-      <c r="E97" s="8" t="s">
-        <v>159</v>
       </c>
       <c r="F97" s="8"/>
       <c r="G97" s="8"/>
     </row>
-    <row r="98" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A98" s="6">
         <v>8</v>
       </c>
       <c r="B98" s="6" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C98" s="10" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="D98" s="8" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E98" s="8" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="F98" s="8"/>
       <c r="G98" s="8"/>
     </row>
-    <row r="99" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A99" s="6">
         <v>8</v>
       </c>
       <c r="B99" s="6" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C99" s="11" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="D99" s="8" t="s">
         <v>51</v>
       </c>
       <c r="E99" s="8" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="F99" s="8"/>
       <c r="G99" s="8"/>
     </row>
-    <row r="100" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A100" s="6">
         <v>8</v>
       </c>
       <c r="B100" s="6" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C100" s="12" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="D100" s="8" t="s">
         <v>57</v>
       </c>
       <c r="E100" s="8" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="F100" s="8"/>
       <c r="G100" s="8"/>
     </row>
-    <row r="101" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A101" s="6">
         <v>8</v>
       </c>
       <c r="B101" s="6" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C101" s="13" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="D101" s="8" t="s">
         <v>61</v>
       </c>
       <c r="E101" s="8" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="F101" s="8"/>
       <c r="G101" s="8"/>
@@ -3556,16 +3562,16 @@
         <v>8</v>
       </c>
       <c r="B102" s="6" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C102" s="9" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="D102" s="8" t="s">
         <v>79</v>
       </c>
       <c r="E102" s="8" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="F102" s="8"/>
       <c r="G102" s="8"/>
@@ -3575,54 +3581,54 @@
         <v>8</v>
       </c>
       <c r="B103" s="6" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C103" s="9" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="D103" s="8" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E103" s="8" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="F103" s="8"/>
       <c r="G103" s="8"/>
     </row>
-    <row r="104" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A104" s="6">
         <v>8</v>
       </c>
       <c r="B104" s="6" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C104" s="7" t="s">
         <v>43</v>
       </c>
       <c r="D104" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="E104" s="8" t="s">
         <v>166</v>
-      </c>
-      <c r="E104" s="8" t="s">
-        <v>167</v>
       </c>
       <c r="F104" s="8"/>
       <c r="G104" s="8"/>
     </row>
-    <row r="105" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A105" s="6">
         <v>9</v>
       </c>
       <c r="B105" s="6" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C105" s="7" t="s">
         <v>43</v>
       </c>
       <c r="D105" s="8" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="E105" s="8" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="F105" s="8"/>
       <c r="G105" s="8"/>
@@ -3632,16 +3638,16 @@
         <v>10</v>
       </c>
       <c r="B106" s="6" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C106" s="9" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="D106" s="8" t="s">
         <v>79</v>
       </c>
       <c r="E106" s="8" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="F106" s="8"/>
       <c r="G106" s="8"/>
@@ -3651,16 +3657,16 @@
         <v>11</v>
       </c>
       <c r="B107" s="6" t="s">
+        <v>171</v>
+      </c>
+      <c r="C107" s="9" t="s">
+        <v>267</v>
+      </c>
+      <c r="D107" s="8" t="s">
         <v>172</v>
       </c>
-      <c r="C107" s="9" t="s">
-        <v>268</v>
-      </c>
-      <c r="D107" s="8" t="s">
+      <c r="E107" s="8" t="s">
         <v>173</v>
-      </c>
-      <c r="E107" s="8" t="s">
-        <v>174</v>
       </c>
       <c r="F107" s="8"/>
       <c r="G107" s="8"/>
@@ -3670,85 +3676,79 @@
         <v>11</v>
       </c>
       <c r="B108" s="6" t="s">
+        <v>171</v>
+      </c>
+      <c r="C108" s="9" t="s">
+        <v>267</v>
+      </c>
+      <c r="D108" s="8" t="s">
         <v>172</v>
       </c>
-      <c r="C108" s="9" t="s">
-        <v>268</v>
-      </c>
-      <c r="D108" s="8" t="s">
-        <v>173</v>
-      </c>
       <c r="E108" s="8" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="F108" s="8"/>
       <c r="G108" s="8"/>
     </row>
-    <row r="109" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A109" s="6">
         <v>12</v>
       </c>
       <c r="B109" s="6" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C109" s="7" t="s">
         <v>43</v>
       </c>
       <c r="D109" s="8" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="E109" s="8" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="F109" s="8"/>
       <c r="G109" s="8"/>
     </row>
-    <row r="110" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A110" s="6">
         <v>13</v>
       </c>
       <c r="B110" s="6" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C110" s="7" t="s">
         <v>43</v>
       </c>
       <c r="D110" s="8" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="E110" s="8" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="F110" s="8"/>
       <c r="G110" s="8"/>
     </row>
-    <row r="111" spans="1:7" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A111" s="6">
         <v>13</v>
       </c>
       <c r="B111" s="6" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C111" s="7" t="s">
         <v>43</v>
       </c>
       <c r="D111" s="8" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="E111" s="8" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="F111" s="8"/>
       <c r="G111" s="8"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G111" xr:uid="{00000000-0001-0000-0100-000000000000}">
-    <filterColumn colId="2">
-      <filters>
-        <filter val="Helen"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:G111" xr:uid="{00000000-0001-0000-0100-000000000000}"/>
   <conditionalFormatting sqref="F2:F111">
     <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
       <formula>"Done"</formula>
@@ -3779,7 +3779,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="18" x14ac:dyDescent="0.2">
       <c r="A1" s="39" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B1" s="39"/>
       <c r="C1" s="39"/>
@@ -3791,21 +3791,21 @@
         <v>37</v>
       </c>
       <c r="B3" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="C3" s="5" t="s">
         <v>182</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="D3" s="5" t="s">
         <v>183</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="E3" s="5" t="s">
         <v>184</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>185</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" s="30" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="B4" s="14" t="s">
         <v>6</v>
@@ -3825,7 +3825,7 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" s="31" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B5" s="14" t="s">
         <v>10</v>
@@ -3845,7 +3845,7 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" s="32" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B6" s="14" t="s">
         <v>14</v>
@@ -3865,7 +3865,7 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" s="33" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="B7" s="14" t="s">
         <v>18</v>
@@ -3885,7 +3885,7 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" s="34" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="B8" s="14" t="s">
         <v>22</v>
@@ -3908,7 +3908,7 @@
         <v>43</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C9" s="14">
         <f>COUNTIF('Daily Tasks'!C:C,"TEAM")</f>
@@ -3916,16 +3916,16 @@
       </c>
       <c r="D9" s="14">
         <f>COUNTIFS('Daily Tasks'!C:C,"TEAM",'Daily Tasks'!F:F,"Done")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E9" s="15">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.125</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" s="16" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B10" s="17"/>
       <c r="C10" s="16">
@@ -3934,16 +3934,16 @@
       </c>
       <c r="D10" s="16">
         <f>SUM(D4:D9)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E10" s="18">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.125</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="18" x14ac:dyDescent="0.2">
       <c r="A12" s="39" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B12" s="39"/>
       <c r="C12" s="39"/>
@@ -3958,13 +3958,13 @@
         <v>36</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="D14" s="5" t="s">
+        <v>183</v>
+      </c>
+      <c r="E14" s="5" t="s">
         <v>184</v>
-      </c>
-      <c r="E14" s="5" t="s">
-        <v>185</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">
@@ -3980,11 +3980,11 @@
       </c>
       <c r="D15" s="14">
         <f>COUNTIFS('Daily Tasks'!A:A,1,'Daily Tasks'!F:F,"Done")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E15" s="15">
         <f t="shared" ref="E15:E27" si="1">IFERROR(D15/C15,0)</f>
-        <v>6.6666666666666666E-2</v>
+        <v>0.13333333333333333</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.2">
@@ -4000,11 +4000,11 @@
       </c>
       <c r="D16" s="14">
         <f>COUNTIFS('Daily Tasks'!A:A,2,'Daily Tasks'!F:F,"Done")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E16" s="15">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>6.6666666666666666E-2</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.2">
@@ -4032,7 +4032,7 @@
         <v>4</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C18" s="14">
         <f>COUNTIF('Daily Tasks'!A:A,4)</f>
@@ -4052,7 +4052,7 @@
         <v>5</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C19" s="14">
         <f>COUNTIF('Daily Tasks'!A:A,5)</f>
@@ -4072,7 +4072,7 @@
         <v>6</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C20" s="14">
         <f>COUNTIF('Daily Tasks'!A:A,6)</f>
@@ -4092,7 +4092,7 @@
         <v>7</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C21" s="14">
         <f>COUNTIF('Daily Tasks'!A:A,7)</f>
@@ -4112,7 +4112,7 @@
         <v>8</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C22" s="14">
         <f>COUNTIF('Daily Tasks'!A:A,8)</f>
@@ -4132,7 +4132,7 @@
         <v>9</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C23" s="14">
         <f>COUNTIF('Daily Tasks'!A:A,9)</f>
@@ -4152,7 +4152,7 @@
         <v>10</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C24" s="14">
         <f>COUNTIF('Daily Tasks'!A:A,10)</f>
@@ -4172,7 +4172,7 @@
         <v>11</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C25" s="14">
         <f>COUNTIF('Daily Tasks'!A:A,11)</f>
@@ -4192,7 +4192,7 @@
         <v>12</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C26" s="14">
         <f>COUNTIF('Daily Tasks'!A:A,12)</f>
@@ -4212,7 +4212,7 @@
         <v>13</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C27" s="14">
         <f>COUNTIF('Daily Tasks'!A:A,13)</f>
@@ -4249,7 +4249,7 @@
   <sheetData>
     <row r="1" spans="1:4" ht="18" x14ac:dyDescent="0.2">
       <c r="A1" s="39" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B1" s="39"/>
       <c r="C1" s="39"/>
@@ -4257,7 +4257,7 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" s="40" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B2" s="40"/>
       <c r="C2" s="40"/>
@@ -4265,13 +4265,13 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" s="5" t="s">
+        <v>191</v>
+      </c>
+      <c r="B4" s="5" t="s">
         <v>192</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="C4" s="5" t="s">
         <v>193</v>
-      </c>
-      <c r="C4" s="5" t="s">
-        <v>194</v>
       </c>
       <c r="D4" s="5" t="s">
         <v>40</v>
@@ -4279,322 +4279,322 @@
     </row>
     <row r="5" spans="1:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="20" t="s">
+        <v>194</v>
+      </c>
+      <c r="B5" s="8" t="s">
         <v>195</v>
       </c>
-      <c r="B5" s="8" t="s">
-        <v>196</v>
-      </c>
       <c r="C5" s="10" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="D5" s="21"/>
     </row>
     <row r="6" spans="1:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="20" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="D6" s="21"/>
     </row>
     <row r="7" spans="1:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="20" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="D7" s="21"/>
     </row>
     <row r="8" spans="1:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="20" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C8" s="12" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="D8" s="21"/>
     </row>
     <row r="9" spans="1:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="20" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="D9" s="21"/>
     </row>
     <row r="10" spans="1:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="20" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C10" s="13" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="D10" s="21"/>
     </row>
     <row r="11" spans="1:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="20" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="D11" s="21"/>
     </row>
     <row r="12" spans="1:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="20" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C12" s="13" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="D12" s="21"/>
     </row>
     <row r="13" spans="1:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="20" t="s">
+        <v>203</v>
+      </c>
+      <c r="B13" s="8" t="s">
         <v>204</v>
       </c>
-      <c r="B13" s="8" t="s">
-        <v>205</v>
-      </c>
       <c r="C13" s="10" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="D13" s="21"/>
     </row>
     <row r="14" spans="1:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="20" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="D14" s="21"/>
     </row>
     <row r="15" spans="1:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="20" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="D15" s="21"/>
     </row>
     <row r="16" spans="1:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="20" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C16" s="10" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="D16" s="21"/>
     </row>
     <row r="17" spans="1:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="20" t="s">
+        <v>208</v>
+      </c>
+      <c r="B17" s="8" t="s">
         <v>209</v>
       </c>
-      <c r="B17" s="8" t="s">
-        <v>210</v>
-      </c>
       <c r="C17" s="11" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="D17" s="21"/>
     </row>
     <row r="18" spans="1:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="20" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C18" s="11" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="D18" s="21"/>
     </row>
     <row r="19" spans="1:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="20" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C19" s="11" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="D19" s="21"/>
     </row>
     <row r="20" spans="1:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="20" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C20" s="11" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="D20" s="21"/>
     </row>
     <row r="21" spans="1:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="20" t="s">
+        <v>213</v>
+      </c>
+      <c r="B21" s="8" t="s">
         <v>214</v>
       </c>
-      <c r="B21" s="8" t="s">
-        <v>215</v>
-      </c>
       <c r="C21" s="12" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="D21" s="21"/>
     </row>
     <row r="22" spans="1:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="20" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C22" s="12" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="D22" s="21"/>
     </row>
     <row r="23" spans="1:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="20" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C23" s="12" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="D23" s="21"/>
     </row>
     <row r="24" spans="1:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="20" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C24" s="12" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="D24" s="21"/>
     </row>
     <row r="25" spans="1:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="20" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C25" s="12" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="D25" s="21"/>
     </row>
     <row r="26" spans="1:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="20" t="s">
+        <v>219</v>
+      </c>
+      <c r="B26" s="8" t="s">
         <v>220</v>
       </c>
-      <c r="B26" s="8" t="s">
-        <v>221</v>
-      </c>
       <c r="C26" s="13" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="D26" s="21"/>
     </row>
     <row r="27" spans="1:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="20" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B27" s="8" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="C27" s="13" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="D27" s="21"/>
     </row>
     <row r="28" spans="1:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="20" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B28" s="8" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="C28" s="13" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="D28" s="21"/>
     </row>
     <row r="29" spans="1:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="20" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B29" s="8" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C29" s="13" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="D29" s="21"/>
     </row>
     <row r="30" spans="1:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="20" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B30" s="8" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="C30" s="13" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="D30" s="21"/>
     </row>
     <row r="31" spans="1:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="20" t="s">
+        <v>225</v>
+      </c>
+      <c r="B31" s="8" t="s">
         <v>226</v>
-      </c>
-      <c r="B31" s="8" t="s">
-        <v>227</v>
       </c>
       <c r="C31" s="7" t="s">
         <v>43</v>
@@ -4603,130 +4603,130 @@
     </row>
     <row r="32" spans="1:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="20" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B32" s="8" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="C32" s="10" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="D32" s="21"/>
     </row>
     <row r="33" spans="1:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="20" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B33" s="8" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="C33" s="10" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="D33" s="21"/>
     </row>
     <row r="34" spans="1:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="20" t="s">
+        <v>229</v>
+      </c>
+      <c r="B34" s="8" t="s">
         <v>230</v>
       </c>
-      <c r="B34" s="8" t="s">
-        <v>231</v>
-      </c>
       <c r="C34" s="9" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="D34" s="21"/>
     </row>
     <row r="35" spans="1:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="20" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B35" s="8" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="C35" s="9" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="D35" s="21"/>
     </row>
     <row r="36" spans="1:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="20" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B36" s="8" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="C36" s="9" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="D36" s="21"/>
     </row>
     <row r="37" spans="1:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="20" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B37" s="8" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C37" s="9" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="D37" s="21"/>
     </row>
     <row r="38" spans="1:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="20" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B38" s="8" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="C38" s="9" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="D38" s="21"/>
     </row>
     <row r="39" spans="1:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="20" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B39" s="8" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="C39" s="9" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="D39" s="21"/>
     </row>
     <row r="40" spans="1:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="20" t="s">
+        <v>236</v>
+      </c>
+      <c r="B40" s="8" t="s">
         <v>237</v>
       </c>
-      <c r="B40" s="8" t="s">
-        <v>238</v>
-      </c>
       <c r="C40" s="9" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="D40" s="21"/>
     </row>
     <row r="41" spans="1:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="20" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="B41" s="8" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C41" s="9" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="D41" s="21"/>
     </row>
     <row r="42" spans="1:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="20" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="B42" s="8" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="C42" s="7" t="s">
         <v>43</v>
@@ -4735,34 +4735,34 @@
     </row>
     <row r="43" spans="1:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="20" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="B43" s="8" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="C43" s="9" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="D43" s="21"/>
     </row>
     <row r="44" spans="1:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="20" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="B44" s="8" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="C44" s="9" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="D44" s="21"/>
     </row>
     <row r="45" spans="1:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="20" t="s">
+        <v>242</v>
+      </c>
+      <c r="B45" s="8" t="s">
         <v>243</v>
-      </c>
-      <c r="B45" s="8" t="s">
-        <v>244</v>
       </c>
       <c r="C45" s="7" t="s">
         <v>43</v>
@@ -4771,10 +4771,10 @@
     </row>
     <row r="46" spans="1:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="20" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B46" s="8" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="C46" s="7" t="s">
         <v>43</v>
@@ -4783,118 +4783,118 @@
     </row>
     <row r="47" spans="1:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="20" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B47" s="8" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="C47" s="10" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="D47" s="21"/>
     </row>
     <row r="48" spans="1:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="20" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B48" s="8" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="C48" s="9" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="D48" s="21"/>
     </row>
     <row r="49" spans="1:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="20" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B49" s="8" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="C49" s="9" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="D49" s="21"/>
     </row>
     <row r="50" spans="1:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="20" t="s">
+        <v>248</v>
+      </c>
+      <c r="B50" s="8" t="s">
         <v>249</v>
       </c>
-      <c r="B50" s="8" t="s">
-        <v>250</v>
-      </c>
       <c r="C50" s="9" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="D50" s="21"/>
     </row>
     <row r="51" spans="1:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="20" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B51" s="8" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="C51" s="9" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="D51" s="21"/>
     </row>
     <row r="52" spans="1:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="20" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B52" s="8" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="C52" s="9" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="D52" s="21"/>
     </row>
     <row r="53" spans="1:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="20" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B53" s="8" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="C53" s="10" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="D53" s="21"/>
     </row>
     <row r="54" spans="1:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="20" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B54" s="8" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="C54" s="9" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="D54" s="21"/>
     </row>
     <row r="55" spans="1:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="20" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B55" s="8" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="C55" s="9" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="D55" s="21"/>
     </row>
     <row r="56" spans="1:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="20" t="s">
+        <v>255</v>
+      </c>
+      <c r="B56" s="8" t="s">
         <v>256</v>
-      </c>
-      <c r="B56" s="8" t="s">
-        <v>257</v>
       </c>
       <c r="C56" s="7" t="s">
         <v>43</v>
@@ -4903,43 +4903,43 @@
     </row>
     <row r="57" spans="1:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="20" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="B57" s="8" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="C57" s="9" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="D57" s="21"/>
     </row>
     <row r="58" spans="1:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="20" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="B58" s="8" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="C58" s="9" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="D58" s="21"/>
     </row>
     <row r="59" spans="1:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="20" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="B59" s="8" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="C59" s="9" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="D59" s="21"/>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A62" s="2" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="B62" s="2" t="str">
         <f>COUNTIF(D5:D59,"Verified") &amp; " of 55"</f>
@@ -4948,7 +4948,7 @@
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A63" s="2" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="B63" s="22">
         <f>COUNTIF(D5:D59,"Verified")/55</f>

</xml_diff>